<commit_message>
Enhance KPI cards, quality section and dashboard formatting
</commit_message>
<xml_diff>
--- a/excel/Daily_Performance_Board.xlsx
+++ b/excel/Daily_Performance_Board.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PROPRIETAIRE\Desktop\data analytics\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PROPRIETAIRE\Desktop\data analytics\daily-performance-board\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAA6E12D-2F87-452C-8EDF-BAFD12BDB294}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA1AB8EC-C475-435C-B25F-A36E6593653E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="10284" firstSheet="2" activeTab="5" xr2:uid="{262B7350-0BCB-4C3E-A161-B1063555A7F0}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="10284" firstSheet="1" activeTab="5" xr2:uid="{262B7350-0BCB-4C3E-A161-B1063555A7F0}"/>
   </bookViews>
   <sheets>
     <sheet name="01_PARAMETRES" sheetId="2" r:id="rId1"/>
@@ -20,10 +20,6 @@
     <sheet name="06_ANALYSE_HEBDO" sheetId="5" r:id="rId5"/>
     <sheet name="05_DASHBOARD_JOUR" sheetId="4" r:id="rId6"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">'03_HISTORIQUE'!$B$4:$B$25</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">'03_HISTORIQUE'!$J$4:$J$25</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -34,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="77">
   <si>
     <t>FormatID</t>
   </si>
@@ -240,9 +236,6 @@
     <t>Écart vs objectif</t>
   </si>
   <si>
-    <t>P</t>
-  </si>
-  <si>
     <t>TAUX DECLASSEMENT</t>
   </si>
   <si>
@@ -259,6 +252,16 @@
   </si>
   <si>
     <t>8h00</t>
+  </si>
+  <si>
+    <t>Objectif qualité atteint</t>
+  </si>
+  <si>
+    <t>Taux de déclassement inférieur à l'objectif de 1,5%
+ Poursuivre les efforts pour maintenir la performance et maintenir les pertes</t>
+  </si>
+  <si>
+    <t>PILOTAGE QUOTIDIEN DES OBJECTIF DE PRODUCTION</t>
   </si>
 </sst>
 </file>
@@ -266,10 +269,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="169" formatCode="0.0%"/>
-    <numFmt numFmtId="171" formatCode="\+#\ ##0;\-#\ ##0"/>
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="\+#\ ##0;\-#\ ##0"/>
   </numFmts>
-  <fonts count="49">
+  <fonts count="51">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -601,8 +604,22 @@
       <name val="Segoe UI Semibold"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="22"/>
+      <color theme="4" tint="-0.499984740745262"/>
+      <name val="Segoe UI Semibold"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="26"/>
+      <color rgb="FF002060"/>
+      <name val="Segoe UI Semibold"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -663,8 +680,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="37">
+  <borders count="44">
     <border>
       <left/>
       <right/>
@@ -712,17 +735,6 @@
       <bottom style="thin">
         <color rgb="FF7030A0"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7030A0"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF7030A0"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -1034,12 +1046,92 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0" tint="-4.9989318521683403E-2"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-4.9989318521683403E-2"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="0" tint="-4.9989318521683403E-2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="0" tint="-4.9989318521683403E-2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0" tint="-4.9989318521683403E-2"/>
+      </right>
+      <top style="thin">
+        <color theme="0" tint="-4.9989318521683403E-2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-4.9989318521683403E-2"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0" tint="-4.9989318521683403E-2"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="0" tint="-4.9989318521683403E-2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="0" tint="-4.9989318521683403E-2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0" tint="-4.9989318521683403E-2"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="0" tint="-4.9989318521683403E-2"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="167">
+  <cellXfs count="185">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1086,7 +1178,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1100,26 +1192,11 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1132,41 +1209,29 @@
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="30" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1177,10 +1242,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1190,10 +1252,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="34" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="34" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="34" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1206,7 +1264,7 @@
     <xf numFmtId="0" fontId="32" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1215,7 +1273,7 @@
     <xf numFmtId="0" fontId="31" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1223,116 +1281,42 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="10" fillId="4" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="10" fillId="4" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="10" fillId="9" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="10" fillId="9" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="10" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="10" fillId="10" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1343,7 +1327,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="34" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1371,17 +1355,169 @@
     <xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="18" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="18" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="10" fillId="10" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="10" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="10" fillId="9" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="10" fillId="9" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="10" fillId="4" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="10" fillId="4" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="35" fillId="6" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="6" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="6" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="18" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="18" fillId="0" borderId="36" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1399,6 +1535,28 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1419,28 +1577,6 @@
         <scheme val="minor"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1483,8 +1619,8 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="6.1642312902995794E-2"/>
-          <c:y val="4.1450380411309343E-2"/>
+          <c:x val="6.0068491792633572E-2"/>
+          <c:y val="3.8803379397712855E-2"/>
           <c:w val="0.81106131138523596"/>
           <c:h val="0.56190903352270838"/>
         </c:manualLayout>
@@ -1496,7 +1632,15 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Objectif</c:v>
+            <c:strRef>
+              <c:f>'05_DASHBOARD_JOUR'!$AF$20</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>OBJECTIF</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:tx>
           <c:spPr>
             <a:ln w="38100" cap="rnd">
@@ -1511,9 +1655,6 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
-          <c:dLbls>
-            <c:delete val="1"/>
-          </c:dLbls>
           <c:cat>
             <c:numRef>
               <c:f>'05_DASHBOARD_JOUR'!$AB$21:$AB$27</c:f>
@@ -1585,7 +1726,15 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:v>Taux</c:v>
+            <c:strRef>
+              <c:f>'05_DASHBOARD_JOUR'!$AE$20</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>TAUX</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
           </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
@@ -1657,6 +1806,36 @@
               </c:ext>
             </c:extLst>
           </c:dLbls>
+          <c:cat>
+            <c:numRef>
+              <c:f>'05_DASHBOARD_JOUR'!$AB$21:$AB$27</c:f>
+              <c:numCache>
+                <c:formatCode>m/d/yyyy</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>46187</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46188</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46189</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>46190</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>46191</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>46192</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>46193</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>'05_DASHBOARD_JOUR'!$AE$21:$AE$27</c:f>
@@ -1695,9 +1874,8 @@
           </c:extLst>
         </c:ser>
         <c:dLbls>
-          <c:dLblPos val="t"/>
           <c:showLegendKey val="0"/>
-          <c:showVal val="1"/>
+          <c:showVal val="0"/>
           <c:showCatName val="0"/>
           <c:showSerName val="0"/>
           <c:showPercent val="0"/>
@@ -2473,7 +2651,7 @@
         <xdr:cNvPr id="4" name="Connecteur droit 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2DAE818D-E29F-494A-95BE-6F21E377DF4F}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000004000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2530,7 +2708,7 @@
         <xdr:cNvPr id="5" name="Connecteur droit 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1F856490-5E7C-4266-B574-91F0DCEC483B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000005000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2587,7 +2765,7 @@
         <xdr:cNvPr id="6" name="Connecteur droit 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{221863E3-2476-4734-AC1C-FBF7F4EC20CA}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000006000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2630,21 +2808,21 @@
     <xdr:from>
       <xdr:col>9</xdr:col>
       <xdr:colOff>15240</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>22</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>23</xdr:col>
       <xdr:colOff>1168400</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>254000</xdr:rowOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>28222</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="17" name="Graphique 16">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0975FFE0-9D90-4FED-9148-B27FEF73968E}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000011000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2680,7 +2858,7 @@
         <xdr:cNvPr id="18" name="Connecteur droit 17">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E2D585E9-45FA-49B2-A91D-CE9775263DE0}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000012000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2737,7 +2915,7 @@
         <xdr:cNvPr id="21" name="Connecteur droit 20">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E2D585E9-45FA-49B2-A91D-CE9775263DE0}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000015000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2794,7 +2972,7 @@
         <xdr:cNvPr id="22" name="Connecteur droit 21">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AEE34D96-F720-4DDB-B283-AC54BCC852B7}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000016000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2833,19 +3011,496 @@
     </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>225779</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>-1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>649114</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>56445</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Graphique 2" descr="Usine">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{11E7F30D-2682-41C5-9776-B4AF1CA2BF0B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId3"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="423335" y="761999"/>
+          <a:ext cx="1636890" cy="1636890"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>169333</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>197556</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1083733</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>237067</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Graphique 7" descr="Mille">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{13843B5C-F323-4C96-B9FE-0485D9863F86}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId5"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="366889" y="16086667"/>
+          <a:ext cx="914400" cy="914400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>141110</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>225778</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1055510</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>265289</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Graphique 11" descr="Graphique à barres avec tendance à la hausse">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5F513E37-01C5-41A0-947F-581FF730810E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId7"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="338666" y="13687778"/>
+          <a:ext cx="914400" cy="914400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>102444</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>74223</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1016844</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>198400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="Graphique 15" descr="Statistiques (droite à gauche)">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9CF07501-A5FE-4DBA-8B66-95A79C625F02}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId9"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="300000" y="12435556"/>
+          <a:ext cx="914400" cy="914400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>167778</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>252444</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1082178</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>914400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="20" name="Graphique 19" descr="Informations">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E52C1437-8E67-4857-B6E8-906D5026E8E7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId11"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10948667" y="18117111"/>
+          <a:ext cx="914400" cy="914400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>366890</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>225776</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>1382889</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>479777</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="24" name="Graphique 23" descr="Calendrier quotidien">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1B16E996-1A6C-4B51-AD4A-ED9620C592FD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId13"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18203334" y="451554"/>
+          <a:ext cx="1806222" cy="1665112"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>197555</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>197555</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1111955</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>237067</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="26" name="Graphique 25" descr="Tendance à la baisse">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2333DCD0-9E2C-436D-9510-AE51E9FB1C87}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId15"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="395111" y="14873111"/>
+          <a:ext cx="914400" cy="914400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>770890</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>121779</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>790223</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>931334</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="30" name="Graphique 29" descr="Trophée">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E828358C-45DA-4F48-857B-CA50BE780429}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId17"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="20865112" y="17958223"/>
+          <a:ext cx="809555" cy="809555"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>355600</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>239889</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1030111</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>914400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="32" name="Graphique 31" descr="Coche">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{45F7068D-8B55-4F81-AEC6-831F9C1247C4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId19"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4800600" y="18045289"/>
+          <a:ext cx="674511" cy="674511"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{52F9BAC2-0E18-415F-8666-72E7B4FDADF6}" name="T_HISTORIQUE" displayName="T_HISTORIQUE" ref="B4:J25" totalsRowShown="0" headerRowDxfId="3" dataDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{52F9BAC2-0E18-415F-8666-72E7B4FDADF6}" name="T_HISTORIQUE" displayName="T_HISTORIQUE" ref="B4:J25" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
   <autoFilter ref="B4:J25" xr:uid="{32BE312E-898B-45B2-8004-6C1E73491403}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{CE6A0F34-42D2-478A-BA3D-F28849BDFB93}" name="DATE" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{D5C7B792-F16F-457B-A674-E56F9EDD8C1C}" name="FORMAT" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{9BB73822-4EE9-45E9-9196-F7C91C16FA41}" name="OBJECTIF_JOUR" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{EF306DB6-6897-439A-8E84-A3FC01ADDB6C}" name="REALISE" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{20A3C998-DA37-46A4-BB0F-6F4D04080E89}" name="DECLASSES" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{6157FD08-7EF3-4FB7-82B8-D5EBFE3588D7}" name="COMMENTAIRE" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{CE6A0F34-42D2-478A-BA3D-F28849BDFB93}" name="DATE" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{D5C7B792-F16F-457B-A674-E56F9EDD8C1C}" name="FORMAT" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{9BB73822-4EE9-45E9-9196-F7C91C16FA41}" name="OBJECTIF_JOUR" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{EF306DB6-6897-439A-8E84-A3FC01ADDB6C}" name="REALISE" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{20A3C998-DA37-46A4-BB0F-6F4D04080E89}" name="DECLASSES" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{6157FD08-7EF3-4FB7-82B8-D5EBFE3588D7}" name="COMMENTAIRE" dataDxfId="3"/>
     <tableColumn id="7" xr3:uid="{2B315B01-FDF9-44B1-8AE6-6A275F99E0B3}" name="ECART" dataDxfId="2">
       <calculatedColumnFormula>T_HISTORIQUE[[#This Row],[REALISE]]-T_HISTORIQUE[[#This Row],[OBJECTIF_JOUR]]</calculatedColumnFormula>
     </tableColumn>
@@ -3265,7 +3920,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="28.8">
+    <row r="23" spans="1:4">
       <c r="A23" s="2" t="s">
         <v>19</v>
       </c>
@@ -3726,7 +4381,7 @@
     <col min="10" max="10" width="27.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:10" ht="28.8">
+    <row r="4" spans="2:10">
       <c r="B4" s="1" t="s">
         <v>35</v>
       </c>
@@ -4462,25 +5117,26 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="3" style="7" customWidth="1"/>
-    <col min="2" max="3" width="11.5546875" style="7"/>
+    <col min="2" max="2" width="17.77734375" style="7" customWidth="1"/>
+    <col min="3" max="3" width="11.5546875" style="7"/>
     <col min="4" max="4" width="21.21875" style="7" customWidth="1"/>
     <col min="5" max="5" width="11.5546875" style="7"/>
     <col min="6" max="6" width="18.33203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="34.44140625" style="77" customWidth="1"/>
+    <col min="7" max="7" width="34.44140625" style="63" customWidth="1"/>
     <col min="8" max="8" width="11.5546875" style="7"/>
     <col min="9" max="9" width="4.6640625" style="7" customWidth="1"/>
     <col min="10" max="11" width="11.5546875" style="7"/>
     <col min="12" max="12" width="16.77734375" style="7" customWidth="1"/>
     <col min="13" max="13" width="11.5546875" style="7"/>
     <col min="14" max="14" width="16.5546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="30.33203125" style="77" customWidth="1"/>
+    <col min="15" max="15" width="30.33203125" style="63" customWidth="1"/>
     <col min="16" max="16" width="11.5546875" style="7"/>
     <col min="17" max="17" width="4.44140625" style="7" customWidth="1"/>
     <col min="18" max="19" width="11.5546875" style="7"/>
     <col min="20" max="20" width="21.5546875" style="7" customWidth="1"/>
     <col min="21" max="21" width="11.5546875" style="7"/>
     <col min="22" max="22" width="15.88671875" style="7" customWidth="1"/>
-    <col min="23" max="23" width="23.88671875" style="7" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="32.109375" style="7" customWidth="1"/>
     <col min="24" max="24" width="17.88671875" style="7" customWidth="1"/>
     <col min="25" max="25" width="63.33203125" style="7" customWidth="1"/>
     <col min="26" max="27" width="11.5546875" style="7"/>
@@ -4547,31 +5203,30 @@
     </row>
     <row r="2" spans="1:35" ht="42.6" customHeight="1">
       <c r="A2" s="8"/>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="154"/>
-      <c r="E2" s="154"/>
-      <c r="F2" s="154"/>
-      <c r="G2" s="155"/>
-      <c r="H2" s="154"/>
-      <c r="I2" s="154"/>
-      <c r="J2" s="154"/>
-      <c r="K2" s="154"/>
-      <c r="L2" s="154"/>
-      <c r="M2" s="154"/>
-      <c r="N2" s="154"/>
-      <c r="O2" s="155"/>
-      <c r="P2" s="154"/>
-      <c r="Q2" s="154"/>
-      <c r="R2" s="154"/>
-      <c r="S2" s="156" t="s">
+      <c r="B2" s="37"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="112"/>
+      <c r="E2" s="112"/>
+      <c r="F2" s="112"/>
+      <c r="G2" s="113"/>
+      <c r="H2" s="112"/>
+      <c r="I2" s="112"/>
+      <c r="J2" s="112"/>
+      <c r="K2" s="112"/>
+      <c r="L2" s="112"/>
+      <c r="M2" s="112"/>
+      <c r="N2" s="112"/>
+      <c r="O2" s="113"/>
+      <c r="P2" s="112"/>
+      <c r="Q2" s="112"/>
+      <c r="R2" s="112"/>
+      <c r="T2" s="115"/>
+      <c r="U2" s="114" t="s">
         <v>35</v>
       </c>
-      <c r="T2" s="157"/>
-      <c r="U2" s="157"/>
-      <c r="V2" s="157"/>
-      <c r="W2" s="78"/>
-      <c r="X2" s="78"/>
+      <c r="V2" s="115"/>
+      <c r="W2" s="64"/>
+      <c r="X2" s="64"/>
       <c r="Y2" s="25"/>
       <c r="Z2" s="7" t="s">
         <v>52</v>
@@ -4633,34 +5288,33 @@
     </row>
     <row r="3" spans="1:35" ht="69.599999999999994" customHeight="1">
       <c r="A3" s="8"/>
-      <c r="B3" s="46"/>
+      <c r="B3" s="37"/>
       <c r="C3" s="8"/>
-      <c r="D3" s="158" t="s">
+      <c r="D3" s="116" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="155"/>
-      <c r="F3" s="154"/>
-      <c r="G3" s="159"/>
-      <c r="H3" s="160"/>
-      <c r="I3" s="154"/>
-      <c r="J3" s="154"/>
-      <c r="K3" s="154"/>
-      <c r="L3" s="154"/>
-      <c r="M3" s="154"/>
-      <c r="N3" s="154"/>
-      <c r="O3" s="155"/>
-      <c r="P3" s="154"/>
-      <c r="Q3" s="154"/>
-      <c r="R3" s="154"/>
-      <c r="S3" s="158" t="str">
+      <c r="E3" s="113"/>
+      <c r="F3" s="112"/>
+      <c r="G3" s="117"/>
+      <c r="H3" s="118"/>
+      <c r="I3" s="112"/>
+      <c r="J3" s="112"/>
+      <c r="K3" s="112"/>
+      <c r="L3" s="112"/>
+      <c r="M3" s="112"/>
+      <c r="N3" s="112"/>
+      <c r="O3" s="113"/>
+      <c r="P3" s="112"/>
+      <c r="Q3" s="112"/>
+      <c r="R3" s="112"/>
+      <c r="T3" s="115"/>
+      <c r="U3" s="116" t="str">
         <f>TEXT(AA2,"jj/mm/aaaa")</f>
         <v>20/06/2026</v>
       </c>
-      <c r="T3" s="157"/>
-      <c r="U3" s="157"/>
-      <c r="V3" s="157"/>
-      <c r="W3" s="78"/>
-      <c r="X3" s="78"/>
+      <c r="V3" s="115"/>
+      <c r="W3" s="64"/>
+      <c r="X3" s="64"/>
       <c r="Y3" s="8"/>
       <c r="Z3" s="7" t="s">
         <v>55</v>
@@ -4718,33 +5372,32 @@
     </row>
     <row r="4" spans="1:35" ht="55.8" customHeight="1">
       <c r="A4" s="8"/>
-      <c r="B4" s="46"/>
+      <c r="B4" s="37"/>
       <c r="C4" s="8"/>
-      <c r="D4" s="154" t="s">
-        <v>66</v>
-      </c>
-      <c r="E4" s="155"/>
-      <c r="F4" s="154"/>
-      <c r="G4" s="159"/>
-      <c r="H4" s="160"/>
-      <c r="I4" s="154"/>
-      <c r="J4" s="154"/>
-      <c r="K4" s="154"/>
-      <c r="L4" s="154"/>
-      <c r="M4" s="154"/>
-      <c r="N4" s="154"/>
-      <c r="O4" s="155"/>
-      <c r="P4" s="154"/>
-      <c r="Q4" s="154"/>
-      <c r="R4" s="154"/>
-      <c r="S4" s="154" t="s">
-        <v>74</v>
-      </c>
-      <c r="T4" s="157"/>
-      <c r="U4" s="157"/>
-      <c r="V4" s="157"/>
-      <c r="W4" s="78"/>
-      <c r="X4" s="78"/>
+      <c r="D4" s="184" t="s">
+        <v>76</v>
+      </c>
+      <c r="E4" s="113"/>
+      <c r="F4" s="112"/>
+      <c r="G4" s="117"/>
+      <c r="H4" s="118"/>
+      <c r="I4" s="112"/>
+      <c r="J4" s="112"/>
+      <c r="K4" s="112"/>
+      <c r="L4" s="112"/>
+      <c r="M4" s="112"/>
+      <c r="N4" s="112"/>
+      <c r="O4" s="113"/>
+      <c r="P4" s="112"/>
+      <c r="Q4" s="112"/>
+      <c r="R4" s="112"/>
+      <c r="T4" s="115"/>
+      <c r="U4" s="181" t="s">
+        <v>73</v>
+      </c>
+      <c r="V4" s="115"/>
+      <c r="W4" s="64"/>
+      <c r="X4" s="64"/>
       <c r="Z4" s="7" t="s">
         <v>56</v>
       </c>
@@ -4793,31 +5446,33 @@
         <v>⬇</v>
       </c>
     </row>
-    <row r="5" spans="1:35" ht="19.8" customHeight="1">
+    <row r="5" spans="1:35" ht="55.8" customHeight="1">
       <c r="A5" s="8"/>
-      <c r="B5" s="46"/>
-      <c r="C5" s="46"/>
-      <c r="D5" s="154"/>
-      <c r="E5" s="154"/>
-      <c r="F5" s="154"/>
-      <c r="G5" s="155"/>
-      <c r="H5" s="154"/>
-      <c r="I5" s="154"/>
-      <c r="J5" s="154"/>
-      <c r="K5" s="154"/>
-      <c r="L5" s="154"/>
-      <c r="M5" s="154"/>
-      <c r="N5" s="154"/>
-      <c r="O5" s="155"/>
-      <c r="P5" s="154"/>
-      <c r="Q5" s="154"/>
-      <c r="R5" s="154"/>
-      <c r="S5" s="157"/>
-      <c r="T5" s="157"/>
-      <c r="U5" s="157"/>
-      <c r="V5" s="157"/>
-      <c r="W5" s="78"/>
-      <c r="X5" s="78"/>
+      <c r="B5" s="37"/>
+      <c r="C5" s="37"/>
+      <c r="D5" s="112" t="s">
+        <v>66</v>
+      </c>
+      <c r="E5" s="112"/>
+      <c r="F5" s="112"/>
+      <c r="G5" s="113"/>
+      <c r="H5" s="112"/>
+      <c r="I5" s="112"/>
+      <c r="J5" s="112"/>
+      <c r="K5" s="112"/>
+      <c r="L5" s="112"/>
+      <c r="M5" s="112"/>
+      <c r="N5" s="112"/>
+      <c r="O5" s="113"/>
+      <c r="P5" s="112"/>
+      <c r="Q5" s="112"/>
+      <c r="R5" s="112"/>
+      <c r="S5" s="115"/>
+      <c r="T5" s="115"/>
+      <c r="U5" s="115"/>
+      <c r="V5" s="115"/>
+      <c r="W5" s="64"/>
+      <c r="X5" s="64"/>
       <c r="Y5" s="8"/>
     </row>
     <row r="6" spans="1:35">
@@ -4846,148 +5501,148 @@
       <c r="W6" s="8"/>
       <c r="X6" s="8"/>
     </row>
-    <row r="7" spans="1:35" s="71" customFormat="1" ht="63" customHeight="1">
-      <c r="A7" s="67"/>
-      <c r="B7" s="93" t="s">
+    <row r="7" spans="1:35" s="58" customFormat="1" ht="63" customHeight="1">
+      <c r="A7" s="57"/>
+      <c r="B7" s="143" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="94"/>
-      <c r="D7" s="94"/>
-      <c r="E7" s="94"/>
-      <c r="F7" s="94"/>
-      <c r="G7" s="94"/>
-      <c r="H7" s="95"/>
-      <c r="I7" s="67"/>
-      <c r="J7" s="109" t="s">
+      <c r="C7" s="144"/>
+      <c r="D7" s="144"/>
+      <c r="E7" s="144"/>
+      <c r="F7" s="144"/>
+      <c r="G7" s="144"/>
+      <c r="H7" s="145"/>
+      <c r="I7" s="57"/>
+      <c r="J7" s="146" t="s">
         <v>5</v>
       </c>
-      <c r="K7" s="108"/>
-      <c r="L7" s="108"/>
-      <c r="M7" s="108"/>
-      <c r="N7" s="108"/>
-      <c r="O7" s="108"/>
-      <c r="P7" s="110"/>
-      <c r="Q7" s="67"/>
-      <c r="R7" s="68" t="s">
+      <c r="K7" s="147"/>
+      <c r="L7" s="147"/>
+      <c r="M7" s="147"/>
+      <c r="N7" s="147"/>
+      <c r="O7" s="147"/>
+      <c r="P7" s="148"/>
+      <c r="Q7" s="57"/>
+      <c r="R7" s="149" t="s">
         <v>7</v>
       </c>
-      <c r="S7" s="69"/>
-      <c r="T7" s="69"/>
-      <c r="U7" s="69"/>
-      <c r="V7" s="69"/>
-      <c r="W7" s="69"/>
-      <c r="X7" s="70"/>
-      <c r="Y7" s="67"/>
+      <c r="S7" s="150"/>
+      <c r="T7" s="150"/>
+      <c r="U7" s="150"/>
+      <c r="V7" s="150"/>
+      <c r="W7" s="150"/>
+      <c r="X7" s="151"/>
+      <c r="Y7" s="57"/>
     </row>
     <row r="8" spans="1:35" s="27" customFormat="1" ht="39.6">
       <c r="A8" s="23"/>
-      <c r="B8" s="96"/>
+      <c r="B8" s="77"/>
       <c r="C8" s="23"/>
       <c r="D8" s="23"/>
       <c r="E8" s="23"/>
       <c r="F8" s="23"/>
-      <c r="G8" s="72"/>
-      <c r="H8" s="97"/>
+      <c r="G8" s="59"/>
+      <c r="H8" s="78"/>
       <c r="I8" s="23"/>
-      <c r="J8" s="111"/>
+      <c r="J8" s="89"/>
       <c r="K8" s="23"/>
       <c r="L8" s="23"/>
       <c r="M8" s="23"/>
       <c r="N8" s="23"/>
-      <c r="O8" s="72"/>
-      <c r="P8" s="112"/>
+      <c r="O8" s="59"/>
+      <c r="P8" s="90"/>
       <c r="Q8" s="23"/>
-      <c r="R8" s="54"/>
+      <c r="R8" s="44"/>
       <c r="S8" s="23"/>
       <c r="T8" s="23"/>
       <c r="U8" s="23"/>
       <c r="V8" s="23"/>
       <c r="W8" s="23"/>
-      <c r="X8" s="55"/>
+      <c r="X8" s="45"/>
       <c r="Y8" s="23"/>
     </row>
     <row r="9" spans="1:35" ht="34.799999999999997">
       <c r="A9" s="8"/>
-      <c r="B9" s="98"/>
-      <c r="C9" s="143" t="s">
+      <c r="B9" s="79"/>
+      <c r="C9" s="152" t="s">
         <v>60</v>
       </c>
-      <c r="D9" s="143"/>
+      <c r="D9" s="152"/>
       <c r="E9" s="8"/>
       <c r="F9" s="8"/>
-      <c r="G9" s="147" t="s">
+      <c r="G9" s="105" t="s">
         <v>61</v>
       </c>
-      <c r="H9" s="99"/>
+      <c r="H9" s="80"/>
       <c r="I9" s="8"/>
-      <c r="J9" s="113"/>
-      <c r="K9" s="142" t="s">
+      <c r="J9" s="91"/>
+      <c r="K9" s="139" t="s">
         <v>60</v>
       </c>
-      <c r="L9" s="142"/>
+      <c r="L9" s="139"/>
       <c r="M9" s="8"/>
       <c r="N9" s="8"/>
-      <c r="O9" s="147" t="s">
+      <c r="O9" s="105" t="s">
         <v>61</v>
       </c>
-      <c r="P9" s="114"/>
+      <c r="P9" s="92"/>
       <c r="Q9" s="8"/>
-      <c r="R9" s="56"/>
+      <c r="R9" s="46"/>
       <c r="S9" s="141" t="s">
         <v>60</v>
       </c>
       <c r="T9" s="141"/>
       <c r="U9" s="8"/>
       <c r="V9" s="8"/>
-      <c r="W9" s="150" t="s">
+      <c r="W9" s="108" t="s">
         <v>61</v>
       </c>
-      <c r="X9" s="57"/>
+      <c r="X9" s="47"/>
       <c r="Y9" s="8"/>
     </row>
     <row r="10" spans="1:35" s="26" customFormat="1" ht="67.8">
       <c r="A10" s="22"/>
-      <c r="B10" s="100"/>
-      <c r="C10" s="49" t="str">
+      <c r="B10" s="81"/>
+      <c r="C10" s="40" t="str">
         <f>AG2</f>
         <v>AVANCE</v>
       </c>
       <c r="D10" s="22"/>
       <c r="E10" s="22"/>
       <c r="F10" s="22"/>
-      <c r="G10" s="148">
+      <c r="G10" s="106">
         <f>AB2</f>
         <v>14000</v>
       </c>
-      <c r="H10" s="101"/>
+      <c r="H10" s="82"/>
       <c r="I10" s="22"/>
-      <c r="J10" s="115"/>
-      <c r="K10" s="48" t="str">
+      <c r="J10" s="93"/>
+      <c r="K10" s="39" t="str">
         <f>AG3</f>
         <v>VIGILANCE</v>
       </c>
       <c r="L10" s="22"/>
       <c r="M10" s="22"/>
       <c r="N10" s="22"/>
-      <c r="O10" s="148">
+      <c r="O10" s="106">
         <f>AB3</f>
         <v>10000</v>
       </c>
-      <c r="P10" s="116"/>
+      <c r="P10" s="94"/>
       <c r="Q10" s="22"/>
-      <c r="R10" s="58"/>
-      <c r="S10" s="47" t="str">
+      <c r="R10" s="48"/>
+      <c r="S10" s="38" t="str">
         <f>AG4</f>
         <v>RETARD</v>
       </c>
       <c r="T10" s="22"/>
       <c r="U10" s="22"/>
       <c r="V10" s="22"/>
-      <c r="W10" s="148">
+      <c r="W10" s="106">
         <f>AB4</f>
         <v>8000</v>
       </c>
-      <c r="X10" s="59"/>
+      <c r="X10" s="49"/>
       <c r="Y10" s="22"/>
       <c r="AA10" s="26">
         <f>SUMIFS(
@@ -5024,284 +5679,278 @@
     </row>
     <row r="11" spans="1:35" s="24" customFormat="1" ht="27">
       <c r="A11" s="20"/>
-      <c r="B11" s="102"/>
+      <c r="B11" s="83"/>
       <c r="C11" s="20"/>
       <c r="D11" s="20"/>
       <c r="E11" s="20"/>
       <c r="F11" s="20"/>
-      <c r="G11" s="149" t="s">
+      <c r="G11" s="107" t="s">
         <v>63</v>
       </c>
-      <c r="H11" s="103"/>
+      <c r="H11" s="84"/>
       <c r="I11" s="20"/>
-      <c r="J11" s="117"/>
+      <c r="J11" s="95"/>
       <c r="K11" s="20"/>
       <c r="L11" s="20"/>
       <c r="M11" s="20"/>
       <c r="N11" s="20"/>
-      <c r="O11" s="149" t="s">
+      <c r="O11" s="107" t="s">
         <v>63</v>
       </c>
-      <c r="P11" s="118"/>
+      <c r="P11" s="96"/>
       <c r="Q11" s="20"/>
-      <c r="R11" s="60"/>
+      <c r="R11" s="50"/>
       <c r="S11" s="20"/>
       <c r="T11" s="20"/>
       <c r="U11" s="20"/>
       <c r="V11" s="20"/>
-      <c r="W11" s="149" t="s">
+      <c r="W11" s="107" t="s">
         <v>63</v>
       </c>
-      <c r="X11" s="61"/>
+      <c r="X11" s="51"/>
       <c r="Y11" s="20"/>
     </row>
-    <row r="12" spans="1:35" s="35" customFormat="1" ht="100.8">
-      <c r="A12" s="34"/>
-      <c r="B12" s="104"/>
-      <c r="C12" s="33" t="str">
+    <row r="12" spans="1:35" s="33" customFormat="1" ht="100.8">
+      <c r="A12" s="32"/>
+      <c r="B12" s="85"/>
+      <c r="C12" s="137" t="str">
         <f>AI2</f>
         <v>⬆</v>
       </c>
-      <c r="D12" s="33"/>
-      <c r="E12" s="34"/>
-      <c r="F12" s="34"/>
-      <c r="G12" s="73"/>
-      <c r="H12" s="105"/>
-      <c r="I12" s="34"/>
-      <c r="J12" s="119"/>
-      <c r="K12" s="45" t="str">
+      <c r="D12" s="137"/>
+      <c r="E12" s="32"/>
+      <c r="F12" s="32"/>
+      <c r="G12" s="60"/>
+      <c r="H12" s="86"/>
+      <c r="I12" s="32"/>
+      <c r="J12" s="97"/>
+      <c r="K12" s="140" t="str">
         <f>AI3</f>
         <v>⚠</v>
       </c>
-      <c r="L12" s="45"/>
-      <c r="M12" s="34"/>
-      <c r="N12" s="34"/>
-      <c r="O12" s="73"/>
-      <c r="P12" s="120"/>
-      <c r="Q12" s="34"/>
-      <c r="R12" s="62"/>
-      <c r="S12" s="36" t="str">
+      <c r="L12" s="140"/>
+      <c r="M12" s="32"/>
+      <c r="N12" s="32"/>
+      <c r="O12" s="60"/>
+      <c r="P12" s="98"/>
+      <c r="Q12" s="32"/>
+      <c r="R12" s="52"/>
+      <c r="S12" s="142" t="str">
         <f>AI4</f>
         <v>⬇</v>
       </c>
-      <c r="T12" s="36"/>
-      <c r="U12" s="34"/>
-      <c r="V12" s="34"/>
-      <c r="W12" s="34"/>
-      <c r="X12" s="63"/>
-    </row>
-    <row r="13" spans="1:35" ht="39.6">
-      <c r="A13" s="8"/>
-      <c r="B13" s="98"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="144" t="s">
+      <c r="T12" s="142"/>
+      <c r="U12" s="32"/>
+      <c r="V12" s="32"/>
+      <c r="W12" s="32"/>
+      <c r="X12" s="53"/>
+    </row>
+    <row r="13" spans="1:35" s="164" customFormat="1" ht="60" customHeight="1">
+      <c r="A13" s="156"/>
+      <c r="B13" s="157"/>
+      <c r="C13" s="153" t="s">
+        <v>67</v>
+      </c>
+      <c r="D13" s="153"/>
+      <c r="E13" s="156"/>
+      <c r="F13" s="156"/>
+      <c r="G13" s="154" t="s">
         <v>39</v>
       </c>
-      <c r="H13" s="99"/>
-      <c r="I13" s="8"/>
-      <c r="J13" s="113"/>
-      <c r="K13" s="8"/>
-      <c r="L13" s="8"/>
-      <c r="M13" s="8"/>
-      <c r="N13" s="8"/>
-      <c r="O13" s="145" t="s">
+      <c r="H13" s="158"/>
+      <c r="I13" s="156"/>
+      <c r="J13" s="159"/>
+      <c r="K13" s="153" t="s">
+        <v>67</v>
+      </c>
+      <c r="L13" s="153"/>
+      <c r="M13" s="156"/>
+      <c r="N13" s="156"/>
+      <c r="O13" s="155" t="s">
         <v>39</v>
       </c>
-      <c r="P13" s="114"/>
-      <c r="Q13" s="8"/>
-      <c r="R13" s="56"/>
-      <c r="S13" s="8"/>
-      <c r="T13" s="8"/>
-      <c r="U13" s="8"/>
-      <c r="V13" s="8"/>
-      <c r="W13" s="146" t="s">
+      <c r="P13" s="160"/>
+      <c r="Q13" s="156"/>
+      <c r="R13" s="161"/>
+      <c r="S13" s="153" t="s">
+        <v>67</v>
+      </c>
+      <c r="T13" s="153"/>
+      <c r="U13" s="156"/>
+      <c r="V13" s="156"/>
+      <c r="W13" s="162" t="s">
         <v>39</v>
       </c>
-      <c r="X13" s="57"/>
-      <c r="Y13" s="8"/>
+      <c r="X13" s="163"/>
+      <c r="Y13" s="156"/>
     </row>
     <row r="14" spans="1:35" s="29" customFormat="1" ht="67.8">
       <c r="A14" s="28"/>
-      <c r="B14" s="106"/>
-      <c r="C14" s="124">
+      <c r="B14" s="87"/>
+      <c r="C14" s="138">
         <f>AE2</f>
         <v>850</v>
       </c>
-      <c r="D14" s="124"/>
+      <c r="D14" s="138"/>
       <c r="E14" s="28"/>
       <c r="F14" s="28"/>
-      <c r="G14" s="125">
+      <c r="G14" s="102">
         <f>AC2</f>
         <v>14850</v>
       </c>
-      <c r="H14" s="107"/>
+      <c r="H14" s="88"/>
       <c r="I14" s="28"/>
-      <c r="J14" s="121"/>
-      <c r="K14" s="124">
+      <c r="J14" s="99"/>
+      <c r="K14" s="138">
         <f>AE3</f>
         <v>-350</v>
       </c>
-      <c r="L14" s="124"/>
+      <c r="L14" s="138"/>
       <c r="M14" s="28"/>
       <c r="N14" s="28"/>
-      <c r="O14" s="125">
+      <c r="O14" s="102">
         <f>AC3</f>
         <v>9650</v>
       </c>
-      <c r="P14" s="122"/>
+      <c r="P14" s="100"/>
       <c r="Q14" s="28"/>
-      <c r="R14" s="64"/>
-      <c r="S14" s="124">
+      <c r="R14" s="54"/>
+      <c r="S14" s="138">
         <f>AE4</f>
         <v>-680</v>
       </c>
-      <c r="T14" s="124"/>
+      <c r="T14" s="138"/>
       <c r="U14" s="28"/>
       <c r="V14" s="28"/>
-      <c r="W14" s="125">
+      <c r="W14" s="102">
         <f>AC4</f>
         <v>7320</v>
       </c>
-      <c r="X14" s="65"/>
-      <c r="Y14" s="125"/>
+      <c r="X14" s="55"/>
+      <c r="Y14" s="102"/>
     </row>
     <row r="15" spans="1:35" s="24" customFormat="1" ht="27">
       <c r="A15" s="20"/>
-      <c r="B15" s="102"/>
-      <c r="C15" s="53" t="s">
-        <v>67</v>
-      </c>
-      <c r="D15" s="53"/>
+      <c r="B15" s="83"/>
       <c r="E15" s="20"/>
       <c r="F15" s="20"/>
-      <c r="G15" s="52" t="s">
+      <c r="G15" s="43" t="s">
         <v>63</v>
       </c>
-      <c r="H15" s="103"/>
+      <c r="H15" s="84"/>
       <c r="I15" s="20"/>
-      <c r="J15" s="117"/>
-      <c r="K15" s="53" t="s">
-        <v>67</v>
-      </c>
-      <c r="L15" s="53"/>
+      <c r="J15" s="95"/>
       <c r="M15" s="20"/>
       <c r="N15" s="20"/>
-      <c r="O15" s="52" t="s">
+      <c r="O15" s="43" t="s">
         <v>63</v>
       </c>
-      <c r="P15" s="123"/>
+      <c r="P15" s="101"/>
       <c r="Q15" s="20"/>
-      <c r="R15" s="60"/>
-      <c r="S15" s="53" t="s">
-        <v>67</v>
-      </c>
-      <c r="T15" s="53"/>
+      <c r="R15" s="50"/>
       <c r="U15" s="20"/>
       <c r="V15" s="20"/>
-      <c r="W15" s="52" t="s">
+      <c r="W15" s="43" t="s">
         <v>63</v>
       </c>
-      <c r="X15" s="66"/>
+      <c r="X15" s="56"/>
       <c r="Y15" s="20"/>
     </row>
     <row r="16" spans="1:35">
       <c r="A16" s="8"/>
-      <c r="B16" s="98"/>
+      <c r="B16" s="79"/>
       <c r="C16" s="8"/>
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
       <c r="F16" s="8"/>
       <c r="G16" s="9"/>
-      <c r="H16" s="99"/>
+      <c r="H16" s="80"/>
       <c r="I16" s="8"/>
-      <c r="J16" s="113"/>
+      <c r="J16" s="91"/>
       <c r="K16" s="8"/>
       <c r="L16" s="8"/>
       <c r="M16" s="8"/>
       <c r="N16" s="8"/>
       <c r="O16" s="9"/>
-      <c r="P16" s="114"/>
+      <c r="P16" s="92"/>
       <c r="Q16" s="8"/>
-      <c r="R16" s="56"/>
+      <c r="R16" s="46"/>
       <c r="S16" s="8"/>
       <c r="T16" s="8"/>
       <c r="U16" s="8"/>
       <c r="V16" s="8"/>
       <c r="W16" s="8"/>
-      <c r="X16" s="57"/>
+      <c r="X16" s="47"/>
       <c r="Y16" s="8"/>
     </row>
     <row r="17" spans="1:32">
       <c r="A17" s="8"/>
-      <c r="B17" s="98"/>
+      <c r="B17" s="79"/>
       <c r="C17" s="8"/>
       <c r="D17" s="8"/>
       <c r="E17" s="8"/>
       <c r="F17" s="8"/>
       <c r="G17" s="9"/>
-      <c r="H17" s="99"/>
+      <c r="H17" s="80"/>
       <c r="I17" s="8"/>
-      <c r="J17" s="113"/>
+      <c r="J17" s="91"/>
       <c r="K17" s="8"/>
       <c r="L17" s="8"/>
       <c r="M17" s="8"/>
       <c r="N17" s="8"/>
       <c r="O17" s="9"/>
-      <c r="P17" s="114"/>
+      <c r="P17" s="92"/>
       <c r="Q17" s="8"/>
-      <c r="R17" s="56"/>
+      <c r="R17" s="46"/>
       <c r="S17" s="8"/>
       <c r="T17" s="8"/>
       <c r="U17" s="8"/>
       <c r="V17" s="8"/>
       <c r="W17" s="8"/>
-      <c r="X17" s="57"/>
+      <c r="X17" s="47"/>
       <c r="Y17" s="8"/>
     </row>
-    <row r="18" spans="1:32" s="140" customFormat="1" ht="38.4">
-      <c r="A18" s="131"/>
-      <c r="B18" s="127" t="s">
-        <v>72</v>
-      </c>
-      <c r="C18" s="128"/>
-      <c r="D18" s="128"/>
-      <c r="E18" s="128"/>
-      <c r="F18" s="129">
+    <row r="18" spans="1:32" s="104" customFormat="1" ht="38.4">
+      <c r="A18" s="103"/>
+      <c r="B18" s="125" t="s">
+        <v>71</v>
+      </c>
+      <c r="C18" s="126"/>
+      <c r="D18" s="126"/>
+      <c r="E18" s="126"/>
+      <c r="F18" s="131">
         <f>AF2</f>
         <v>1.0607142857142857</v>
       </c>
-      <c r="G18" s="129"/>
-      <c r="H18" s="130"/>
-      <c r="I18" s="131"/>
-      <c r="J18" s="132" t="s">
-        <v>72</v>
-      </c>
-      <c r="K18" s="133"/>
-      <c r="L18" s="133"/>
-      <c r="M18" s="133"/>
-      <c r="N18" s="134">
+      <c r="G18" s="131"/>
+      <c r="H18" s="132"/>
+      <c r="I18" s="103"/>
+      <c r="J18" s="135" t="s">
+        <v>71</v>
+      </c>
+      <c r="K18" s="136"/>
+      <c r="L18" s="136"/>
+      <c r="M18" s="136"/>
+      <c r="N18" s="129">
         <f>AF3</f>
         <v>0.96499999999999997</v>
       </c>
-      <c r="O18" s="134"/>
-      <c r="P18" s="135"/>
-      <c r="Q18" s="131"/>
-      <c r="R18" s="136" t="s">
-        <v>72</v>
-      </c>
-      <c r="S18" s="137"/>
-      <c r="T18" s="137"/>
-      <c r="U18" s="137"/>
-      <c r="V18" s="138">
+      <c r="O18" s="129"/>
+      <c r="P18" s="130"/>
+      <c r="Q18" s="103"/>
+      <c r="R18" s="133" t="s">
+        <v>71</v>
+      </c>
+      <c r="S18" s="134"/>
+      <c r="T18" s="134"/>
+      <c r="U18" s="134"/>
+      <c r="V18" s="127">
         <f>AF4</f>
         <v>0.91500000000000004</v>
       </c>
-      <c r="W18" s="138"/>
-      <c r="X18" s="139"/>
-      <c r="Y18" s="131"/>
+      <c r="W18" s="127"/>
+      <c r="X18" s="128"/>
+      <c r="Y18" s="103"/>
     </row>
     <row r="19" spans="1:32" ht="60.6" customHeight="1">
       <c r="A19" s="8"/>
@@ -5332,31 +5981,31 @@
     </row>
     <row r="20" spans="1:32" ht="38.4">
       <c r="A20" s="8"/>
-      <c r="B20" s="38"/>
-      <c r="C20" s="126" t="s">
+      <c r="B20" s="166"/>
+      <c r="C20" s="167" t="s">
         <v>36</v>
       </c>
-      <c r="D20" s="80"/>
-      <c r="E20" s="80"/>
-      <c r="F20" s="80"/>
-      <c r="G20" s="81"/>
-      <c r="H20" s="39"/>
-      <c r="I20" s="40"/>
-      <c r="J20" s="50"/>
-      <c r="K20" s="51"/>
-      <c r="L20" s="40"/>
-      <c r="M20" s="51"/>
-      <c r="N20" s="51"/>
-      <c r="O20" s="75"/>
-      <c r="P20" s="51"/>
-      <c r="Q20" s="51"/>
-      <c r="R20" s="51"/>
-      <c r="S20" s="40"/>
-      <c r="T20" s="40"/>
-      <c r="U20" s="40"/>
-      <c r="V20" s="40"/>
-      <c r="W20" s="40"/>
-      <c r="X20" s="41"/>
+      <c r="D20" s="168"/>
+      <c r="E20" s="168"/>
+      <c r="F20" s="168"/>
+      <c r="G20" s="169"/>
+      <c r="H20" s="170"/>
+      <c r="I20" s="34"/>
+      <c r="J20" s="41"/>
+      <c r="K20" s="42"/>
+      <c r="L20" s="34"/>
+      <c r="M20" s="42"/>
+      <c r="N20" s="42"/>
+      <c r="O20" s="62"/>
+      <c r="P20" s="42"/>
+      <c r="Q20" s="42"/>
+      <c r="R20" s="42"/>
+      <c r="S20" s="34"/>
+      <c r="T20" s="34"/>
+      <c r="U20" s="34"/>
+      <c r="V20" s="34"/>
+      <c r="W20" s="34"/>
+      <c r="X20" s="35"/>
       <c r="Y20" s="8"/>
       <c r="AB20" s="2" t="s">
         <v>35</v>
@@ -5374,22 +6023,24 @@
         <v>61</v>
       </c>
     </row>
-    <row r="21" spans="1:32" ht="29.4">
+    <row r="21" spans="1:32" ht="32.4">
       <c r="A21" s="8"/>
-      <c r="B21" s="42"/>
-      <c r="C21" s="79" t="s">
+      <c r="B21" s="171"/>
+      <c r="C21" s="65" t="s">
         <v>65</v>
       </c>
-      <c r="D21" s="79"/>
-      <c r="E21" s="79"/>
-      <c r="F21" s="79"/>
-      <c r="G21" s="82"/>
-      <c r="H21" s="32"/>
+      <c r="D21" s="65"/>
+      <c r="E21" s="65"/>
+      <c r="F21" s="65"/>
+      <c r="G21" s="66"/>
+      <c r="H21" s="172"/>
       <c r="I21" s="8"/>
       <c r="J21" s="8"/>
       <c r="K21" s="8"/>
       <c r="L21" s="8"/>
-      <c r="M21" s="8"/>
+      <c r="M21" s="31" t="s">
+        <v>62</v>
+      </c>
       <c r="N21" s="8"/>
       <c r="O21" s="9"/>
       <c r="P21" s="8"/>
@@ -5400,7 +6051,7 @@
       <c r="U21" s="8"/>
       <c r="V21" s="8"/>
       <c r="W21" s="8"/>
-      <c r="X21" s="43"/>
+      <c r="X21" s="36"/>
       <c r="Y21" s="8"/>
       <c r="AB21" s="17">
         <v>46187</v>
@@ -5430,22 +6081,19 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:32" ht="32.4">
+    <row r="22" spans="1:32" ht="29.4">
       <c r="A22" s="8"/>
-      <c r="B22" s="89"/>
+      <c r="B22" s="173"/>
       <c r="C22" s="30"/>
       <c r="D22" s="30"/>
       <c r="E22" s="30"/>
       <c r="F22" s="21"/>
-      <c r="G22" s="90"/>
-      <c r="H22" s="21"/>
+      <c r="G22" s="74"/>
+      <c r="H22" s="165"/>
       <c r="I22" s="8"/>
       <c r="J22" s="8"/>
       <c r="K22" s="8"/>
       <c r="L22" s="8"/>
-      <c r="M22" s="31" t="s">
-        <v>62</v>
-      </c>
       <c r="N22" s="8"/>
       <c r="O22" s="9"/>
       <c r="P22" s="8"/>
@@ -5456,7 +6104,7 @@
       <c r="U22" s="8"/>
       <c r="V22" s="8"/>
       <c r="W22" s="8"/>
-      <c r="X22" s="43"/>
+      <c r="X22" s="36"/>
       <c r="Y22" s="8"/>
       <c r="Z22"/>
       <c r="AA22"/>
@@ -5490,13 +6138,13 @@
     </row>
     <row r="23" spans="1:32" ht="29.4">
       <c r="A23" s="8"/>
-      <c r="B23" s="89"/>
+      <c r="B23" s="173"/>
       <c r="C23" s="30"/>
       <c r="D23" s="30"/>
       <c r="E23" s="30"/>
       <c r="F23" s="21"/>
-      <c r="G23" s="90"/>
-      <c r="H23" s="21"/>
+      <c r="G23" s="74"/>
+      <c r="H23" s="165"/>
       <c r="I23" s="8"/>
       <c r="J23" s="8"/>
       <c r="K23" s="8"/>
@@ -5512,7 +6160,7 @@
       <c r="U23" s="8"/>
       <c r="V23" s="8"/>
       <c r="W23" s="8"/>
-      <c r="X23" s="43"/>
+      <c r="X23" s="36"/>
       <c r="Y23" s="8"/>
       <c r="Z23"/>
       <c r="AA23"/>
@@ -5546,14 +6194,14 @@
     </row>
     <row r="24" spans="1:32" ht="61.8" customHeight="1">
       <c r="A24" s="8"/>
-      <c r="B24" s="89"/>
-      <c r="C24" s="161" t="s">
-        <v>71</v>
-      </c>
-      <c r="D24" s="162"/>
-      <c r="E24" s="162"/>
-      <c r="F24" s="163"/>
-      <c r="G24" s="164">
+      <c r="B24" s="173"/>
+      <c r="C24" s="119" t="s">
+        <v>70</v>
+      </c>
+      <c r="D24" s="120"/>
+      <c r="E24" s="120"/>
+      <c r="F24" s="121"/>
+      <c r="G24" s="122">
         <f>SUMIFS(
 T_HISTORIQUE[DECLASSES],
 T_HISTORIQUE[DATE],
@@ -5561,7 +6209,7 @@
 )</f>
         <v>244</v>
       </c>
-      <c r="H24" s="21"/>
+      <c r="H24" s="165"/>
       <c r="I24" s="8"/>
       <c r="J24" s="8"/>
       <c r="K24" s="8"/>
@@ -5577,10 +6225,8 @@
       <c r="U24" s="8"/>
       <c r="V24" s="8"/>
       <c r="W24" s="8"/>
-      <c r="X24" s="43"/>
-      <c r="Y24" s="8" t="s">
-        <v>68</v>
-      </c>
+      <c r="X24" s="36"/>
+      <c r="Y24" s="8"/>
       <c r="Z24"/>
       <c r="AA24"/>
       <c r="AB24" s="17">
@@ -5613,13 +6259,13 @@
     </row>
     <row r="25" spans="1:32" ht="24" customHeight="1">
       <c r="A25" s="8"/>
-      <c r="B25" s="89"/>
+      <c r="B25" s="173"/>
       <c r="C25" s="30"/>
       <c r="D25" s="30"/>
       <c r="E25" s="30"/>
       <c r="F25" s="21"/>
-      <c r="G25" s="74"/>
-      <c r="H25" s="21"/>
+      <c r="G25" s="61"/>
+      <c r="H25" s="165"/>
       <c r="I25" s="8"/>
       <c r="J25" s="8"/>
       <c r="K25" s="8"/>
@@ -5635,7 +6281,7 @@
       <c r="U25" s="8"/>
       <c r="V25" s="8"/>
       <c r="W25" s="8"/>
-      <c r="X25" s="43"/>
+      <c r="X25" s="36"/>
       <c r="Y25" s="8"/>
       <c r="Z25"/>
       <c r="AA25"/>
@@ -5669,14 +6315,14 @@
     </row>
     <row r="26" spans="1:32" ht="67.8">
       <c r="A26" s="8"/>
-      <c r="B26" s="89"/>
-      <c r="C26" s="162" t="s">
-        <v>70</v>
-      </c>
-      <c r="D26" s="162"/>
-      <c r="E26" s="162"/>
-      <c r="F26" s="163"/>
-      <c r="G26" s="165">
+      <c r="B26" s="173"/>
+      <c r="C26" s="120" t="s">
+        <v>69</v>
+      </c>
+      <c r="D26" s="120"/>
+      <c r="E26" s="120"/>
+      <c r="F26" s="121"/>
+      <c r="G26" s="123">
         <f>SUMIFS(
 T_HISTORIQUE[REALISE],
 T_HISTORIQUE[DATE],
@@ -5684,7 +6330,7 @@
 )</f>
         <v>31820</v>
       </c>
-      <c r="H26" s="21"/>
+      <c r="H26" s="165"/>
       <c r="I26" s="8"/>
       <c r="J26" s="8"/>
       <c r="K26" s="8"/>
@@ -5700,7 +6346,7 @@
       <c r="U26" s="8"/>
       <c r="V26" s="8"/>
       <c r="W26" s="8"/>
-      <c r="X26" s="43"/>
+      <c r="X26" s="36"/>
       <c r="Y26" s="8"/>
       <c r="Z26"/>
       <c r="AA26"/>
@@ -5734,13 +6380,13 @@
     </row>
     <row r="27" spans="1:32" ht="27.6" customHeight="1">
       <c r="A27" s="8"/>
-      <c r="B27" s="89"/>
+      <c r="B27" s="173"/>
       <c r="C27" s="30"/>
       <c r="D27" s="30"/>
       <c r="E27" s="30"/>
       <c r="F27" s="21"/>
-      <c r="G27" s="74"/>
-      <c r="H27" s="21"/>
+      <c r="G27" s="61"/>
+      <c r="H27" s="165"/>
       <c r="I27" s="8"/>
       <c r="J27" s="8"/>
       <c r="K27" s="8"/>
@@ -5756,7 +6402,7 @@
       <c r="U27" s="8"/>
       <c r="V27" s="8"/>
       <c r="W27" s="8"/>
-      <c r="X27" s="43"/>
+      <c r="X27" s="36"/>
       <c r="Y27" s="8"/>
       <c r="AB27" s="17">
         <v>46193</v>
@@ -5788,18 +6434,18 @@
     </row>
     <row r="28" spans="1:32" ht="67.8">
       <c r="A28" s="8"/>
-      <c r="B28" s="89"/>
-      <c r="C28" s="161" t="s">
-        <v>69</v>
-      </c>
-      <c r="D28" s="162"/>
-      <c r="E28" s="162"/>
-      <c r="F28" s="163"/>
-      <c r="G28" s="166">
+      <c r="B28" s="173"/>
+      <c r="C28" s="119" t="s">
+        <v>68</v>
+      </c>
+      <c r="D28" s="120"/>
+      <c r="E28" s="120"/>
+      <c r="F28" s="121"/>
+      <c r="G28" s="124">
         <f>IFERROR(AA10/AB10,0)</f>
         <v>7.668133249528598E-3</v>
       </c>
-      <c r="H28" s="21"/>
+      <c r="H28" s="165"/>
       <c r="I28" s="8"/>
       <c r="J28" s="8"/>
       <c r="K28" s="8"/>
@@ -5815,7 +6461,7 @@
       <c r="U28" s="8"/>
       <c r="V28" s="8"/>
       <c r="W28" s="8"/>
-      <c r="X28" s="43"/>
+      <c r="X28" s="36"/>
       <c r="Y28" s="8"/>
       <c r="AB28" s="17">
         <v>46194</v>
@@ -5847,13 +6493,13 @@
     </row>
     <row r="29" spans="1:32" ht="25.8" customHeight="1">
       <c r="A29" s="8"/>
-      <c r="B29" s="89"/>
+      <c r="B29" s="173"/>
       <c r="C29" s="30"/>
       <c r="D29" s="30"/>
       <c r="E29" s="30"/>
       <c r="F29" s="21"/>
-      <c r="G29" s="74"/>
-      <c r="H29" s="21"/>
+      <c r="G29" s="61"/>
+      <c r="H29" s="165"/>
       <c r="I29" s="8"/>
       <c r="J29" s="8"/>
       <c r="K29" s="8"/>
@@ -5869,7 +6515,7 @@
       <c r="U29" s="8"/>
       <c r="V29" s="8"/>
       <c r="W29" s="8"/>
-      <c r="X29" s="43"/>
+      <c r="X29" s="36"/>
       <c r="AB29" s="17">
         <v>46195</v>
       </c>
@@ -5900,18 +6546,18 @@
     </row>
     <row r="30" spans="1:32" ht="67.8">
       <c r="A30" s="8"/>
-      <c r="B30" s="89"/>
-      <c r="C30" s="162" t="s">
+      <c r="B30" s="173"/>
+      <c r="C30" s="120" t="s">
         <v>61</v>
       </c>
-      <c r="D30" s="162"/>
-      <c r="E30" s="162"/>
-      <c r="F30" s="163"/>
-      <c r="G30" s="164" t="str">
+      <c r="D30" s="120"/>
+      <c r="E30" s="120"/>
+      <c r="F30" s="121"/>
+      <c r="G30" s="122" t="str">
         <f>"≤ "&amp;TEXT(1.5%,"0,00%")</f>
         <v>≤ 1,50%</v>
       </c>
-      <c r="H30" s="21"/>
+      <c r="H30" s="165"/>
       <c r="I30" s="8"/>
       <c r="J30" s="8"/>
       <c r="K30" s="8"/>
@@ -5927,7 +6573,7 @@
       <c r="U30" s="8"/>
       <c r="V30" s="8"/>
       <c r="W30" s="8"/>
-      <c r="X30" s="43"/>
+      <c r="X30" s="36"/>
       <c r="AB30" s="17">
         <v>46196</v>
       </c>
@@ -5958,13 +6604,13 @@
     </row>
     <row r="31" spans="1:32" ht="29.4">
       <c r="A31" s="8"/>
-      <c r="B31" s="89"/>
-      <c r="C31" s="30"/>
-      <c r="D31" s="30"/>
-      <c r="E31" s="30"/>
-      <c r="F31" s="21"/>
-      <c r="G31" s="83"/>
-      <c r="H31" s="21"/>
+      <c r="B31" s="174"/>
+      <c r="C31" s="175"/>
+      <c r="D31" s="175"/>
+      <c r="E31" s="175"/>
+      <c r="F31" s="176"/>
+      <c r="G31" s="177"/>
+      <c r="H31" s="178"/>
       <c r="I31" s="8"/>
       <c r="J31" s="8"/>
       <c r="K31" s="8"/>
@@ -5980,7 +6626,7 @@
       <c r="U31" s="8"/>
       <c r="V31" s="8"/>
       <c r="W31" s="8"/>
-      <c r="X31" s="43"/>
+      <c r="X31" s="36"/>
       <c r="AB31" s="17">
         <v>46197</v>
       </c>
@@ -6011,12 +6657,12 @@
     </row>
     <row r="32" spans="1:32" ht="29.4">
       <c r="A32" s="8"/>
-      <c r="B32" s="89"/>
+      <c r="B32" s="73"/>
       <c r="C32" s="21"/>
       <c r="D32" s="21"/>
       <c r="E32" s="21"/>
       <c r="F32" s="21"/>
-      <c r="G32" s="90"/>
+      <c r="G32" s="74"/>
       <c r="H32" s="21"/>
       <c r="I32" s="8"/>
       <c r="J32" s="8"/>
@@ -6033,7 +6679,7 @@
       <c r="U32" s="8"/>
       <c r="V32" s="8"/>
       <c r="W32" s="8"/>
-      <c r="X32" s="43"/>
+      <c r="X32" s="36"/>
       <c r="AB32" s="17">
         <v>46198</v>
       </c>
@@ -6062,14 +6708,14 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:32" ht="29.4">
+    <row r="33" spans="1:32" ht="27.6" customHeight="1">
       <c r="A33" s="8"/>
-      <c r="B33" s="89"/>
+      <c r="B33" s="73"/>
       <c r="C33" s="30"/>
       <c r="D33" s="30"/>
       <c r="E33" s="30"/>
       <c r="F33" s="21"/>
-      <c r="G33" s="83"/>
+      <c r="G33" s="67"/>
       <c r="H33" s="21"/>
       <c r="I33" s="8"/>
       <c r="J33" s="8"/>
@@ -6086,7 +6732,7 @@
       <c r="U33" s="8"/>
       <c r="V33" s="8"/>
       <c r="W33" s="8"/>
-      <c r="X33" s="43"/>
+      <c r="X33" s="36"/>
       <c r="AB33" s="17">
         <v>46199</v>
       </c>
@@ -6115,16 +6761,16 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:32" ht="20.399999999999999">
+    <row r="34" spans="1:32" ht="20.399999999999999" hidden="1">
       <c r="A34" s="8"/>
-      <c r="B34" s="86"/>
-      <c r="C34" s="91"/>
-      <c r="D34" s="91"/>
-      <c r="E34" s="91"/>
-      <c r="F34" s="91"/>
-      <c r="G34" s="92"/>
-      <c r="H34" s="87"/>
-      <c r="I34" s="87"/>
+      <c r="B34" s="70"/>
+      <c r="C34" s="75"/>
+      <c r="D34" s="75"/>
+      <c r="E34" s="75"/>
+      <c r="F34" s="75"/>
+      <c r="G34" s="76"/>
+      <c r="H34" s="71"/>
+      <c r="I34" s="71"/>
       <c r="J34" s="8"/>
       <c r="K34" s="8"/>
       <c r="L34" s="8"/>
@@ -6139,7 +6785,7 @@
       <c r="U34" s="8"/>
       <c r="V34" s="8"/>
       <c r="W34" s="8"/>
-      <c r="X34" s="43"/>
+      <c r="X34" s="36"/>
       <c r="AB34" s="17">
         <v>46200</v>
       </c>
@@ -6168,38 +6814,42 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:32" ht="52.2">
+    <row r="35" spans="1:32" ht="85.8" customHeight="1">
       <c r="A35" s="8"/>
-      <c r="B35" s="151"/>
-      <c r="C35" s="152" t="s">
-        <v>73</v>
-      </c>
-      <c r="D35" s="85"/>
-      <c r="E35" s="85"/>
-      <c r="F35" s="84"/>
-      <c r="G35" s="153" t="str">
+      <c r="B35" s="109"/>
+      <c r="C35" s="110" t="s">
+        <v>72</v>
+      </c>
+      <c r="D35" s="69"/>
+      <c r="E35" s="69"/>
+      <c r="F35" s="68"/>
+      <c r="G35" s="111" t="str">
         <f>IF(AC10&lt;=1.5%,"CONFORME",
 IF(AC10&lt;=2%,"SURVEILLANCE",
 "ACTION"))</f>
         <v>CONFORME</v>
       </c>
-      <c r="H35" s="84"/>
-      <c r="I35" s="88"/>
-      <c r="J35" s="37"/>
-      <c r="K35" s="37"/>
-      <c r="L35" s="37"/>
-      <c r="M35" s="37"/>
-      <c r="N35" s="37"/>
-      <c r="O35" s="76"/>
-      <c r="P35" s="37"/>
-      <c r="Q35" s="37"/>
-      <c r="R35" s="37"/>
-      <c r="S35" s="37"/>
-      <c r="T35" s="37"/>
-      <c r="U35" s="37"/>
-      <c r="V35" s="37"/>
-      <c r="W35" s="37"/>
-      <c r="X35" s="44"/>
+      <c r="H35" s="68"/>
+      <c r="I35" s="72"/>
+      <c r="J35" s="179"/>
+      <c r="K35" s="179"/>
+      <c r="L35" s="179"/>
+      <c r="M35" s="182" t="s">
+        <v>75</v>
+      </c>
+      <c r="N35" s="182"/>
+      <c r="O35" s="182"/>
+      <c r="P35" s="182"/>
+      <c r="Q35" s="182"/>
+      <c r="R35" s="182"/>
+      <c r="S35" s="182"/>
+      <c r="T35" s="182"/>
+      <c r="U35" s="179"/>
+      <c r="V35" s="179"/>
+      <c r="W35" s="183" t="s">
+        <v>74</v>
+      </c>
+      <c r="X35" s="180"/>
       <c r="AB35" s="17">
         <v>46201</v>
       </c>
@@ -6339,21 +6989,8 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="21">
-    <mergeCell ref="B18:E18"/>
-    <mergeCell ref="V18:X18"/>
-    <mergeCell ref="N18:P18"/>
-    <mergeCell ref="F18:H18"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="K15:L15"/>
-    <mergeCell ref="S15:T15"/>
-    <mergeCell ref="R18:U18"/>
-    <mergeCell ref="J18:M18"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="K9:L9"/>
-    <mergeCell ref="K12:L12"/>
-    <mergeCell ref="K14:L14"/>
+  <mergeCells count="22">
+    <mergeCell ref="M35:T35"/>
     <mergeCell ref="S9:T9"/>
     <mergeCell ref="S12:T12"/>
     <mergeCell ref="S14:T14"/>
@@ -6361,9 +6998,23 @@
     <mergeCell ref="J7:P7"/>
     <mergeCell ref="R7:X7"/>
     <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="K12:L12"/>
+    <mergeCell ref="K14:L14"/>
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="V18:X18"/>
+    <mergeCell ref="N18:P18"/>
+    <mergeCell ref="F18:H18"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="K13:L13"/>
+    <mergeCell ref="S13:T13"/>
+    <mergeCell ref="R18:U18"/>
+    <mergeCell ref="J18:M18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="32" fitToWidth="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="30" fitToWidth="0" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>